<commit_message>
OMIE: caché de días descargados + reintentos (evita perder datos si la web falla)
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1038,14 +1038,11 @@
       <c r="B16" s="12" t="n">
         <v>37.99</v>
       </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E16" s="17">
-        <f>AVERAGE(E6:E15)</f>
-        <v/>
+      <c r="D16" s="13" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>60.44</v>
       </c>
       <c r="J16" s="14">
         <f>A52</f>
@@ -1063,10 +1060,14 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E17" s="17">
+        <f>AVERAGE(E6:E16)</f>
+        <v/>
       </c>
       <c r="J17" s="14">
         <f>A53</f>
@@ -1084,13 +1085,18 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
       <c r="K18" s="20">
-        <f>E16</f>
+        <f>E17</f>
         <v/>
       </c>
     </row>
@@ -1443,7 +1449,7 @@
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="D18:H18"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1453,7 +1459,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E15">
+  <conditionalFormatting sqref="E6:E16">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1511,7 +1517,7 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1543,7 +1549,7 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>55.79</v>
+        <v>57.9</v>
       </c>
       <c r="C6" s="26" t="n">
         <v>1</v>
@@ -1561,7 +1567,7 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>54.33</v>
+        <v>57.85</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>0</v>
@@ -1579,7 +1585,7 @@
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>54</v>
+        <v>59.45</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>0</v>
@@ -1597,7 +1603,7 @@
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>54.1</v>
+        <v>57.47</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>3</v>
@@ -1615,7 +1621,7 @@
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>51.32</v>
+        <v>56.64</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>3</v>
@@ -1633,7 +1639,7 @@
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>37.5</v>
+        <v>40.05</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>3</v>
@@ -1646,7 +1652,7 @@
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>35.38</v>
+        <v>37.57</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>2</v>
@@ -1659,7 +1665,7 @@
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>36.44</v>
+        <v>38.81</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>0</v>
@@ -1672,7 +1678,7 @@
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>53.4</v>
+        <v>57.65</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>0</v>
@@ -1685,7 +1691,7 @@
         </is>
       </c>
       <c r="B15" s="25" t="n">
-        <v>39.75</v>
+        <v>42.78</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0</v>
@@ -1698,7 +1704,7 @@
         </is>
       </c>
       <c r="B16" s="25" t="n">
-        <v>28.63</v>
+        <v>29.97</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>0</v>
@@ -1737,7 +1743,7 @@
         </is>
       </c>
       <c r="B20" s="31">
-        <f>MIBGAS_Spot!E16</f>
+        <f>MIBGAS_Spot!E17</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-11
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIBGAS_Spot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Futuros" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Indice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MIBGAS_Spot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Futuros" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-12
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -205,14 +205,14 @@
     <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1066,10 +1066,10 @@
       <c r="B17" s="12" t="n">
         <v>34.54</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="13" t="n">
         <v>46246</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="12" t="n">
         <v>59.05</v>
       </c>
       <c r="J17" s="14">
@@ -1088,22 +1088,19 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E18" s="19">
-        <f>AVERAGE(E6:E17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="inlineStr">
+      <c r="D18" s="16" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E18" s="17" t="n">
+        <v>60.45</v>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="K18" s="21">
-        <f>E18</f>
+      <c r="K18" s="19">
+        <f>E19</f>
         <v/>
       </c>
     </row>
@@ -1114,10 +1111,14 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E19" s="21">
+        <f>AVERAGE(E6:E18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1127,6 +1128,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1457,9 +1463,9 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D20:H20"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D19:H19"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
@@ -1471,7 +1477,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E17">
+  <conditionalFormatting sqref="E6:E18">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1529,7 +1535,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1561,7 +1567,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>60.47</v>
+        <v>60.34</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1579,7 +1585,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>59.12</v>
+        <v>60.05</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1597,7 +1603,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>58.05</v>
+        <v>59.45</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1615,7 +1621,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>58.1</v>
+        <v>59.58</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1633,7 +1639,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>54.69</v>
+        <v>56.84</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>38.8</v>
+        <v>39.48</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1664,7 +1670,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>36.36</v>
+        <v>37.04</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1677,7 +1683,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>37.57</v>
+        <v>38.25</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1690,7 +1696,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>56.43</v>
+        <v>58.23</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1703,7 +1709,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>41.43</v>
+        <v>42.55</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1716,7 +1722,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>29.38</v>
+        <v>29.58</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1755,7 +1761,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E18</f>
+        <f>MIBGAS_Spot!E19</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-13
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -199,16 +199,16 @@
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1088,19 +1088,19 @@
       <c r="B18" s="12" t="n">
         <v>29.92</v>
       </c>
-      <c r="D18" s="16" t="n">
+      <c r="D18" s="13" t="n">
         <v>46247</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="12" t="n">
         <v>60.45</v>
       </c>
-      <c r="J18" s="18" t="inlineStr">
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="K18" s="19">
-        <f>E19</f>
+      <c r="K18" s="17">
+        <f>E20</f>
         <v/>
       </c>
     </row>
@@ -1111,14 +1111,11 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E19" s="21">
-        <f>AVERAGE(E6:E18)</f>
-        <v/>
+      <c r="D19" s="18" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>60.77</v>
       </c>
     </row>
     <row r="20">
@@ -1128,10 +1125,14 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E20" s="21">
+        <f>AVERAGE(E6:E19)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1141,6 +1142,11 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1462,8 +1468,8 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D21:H21"/>
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D20:H20"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
@@ -1477,7 +1483,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E18">
+  <conditionalFormatting sqref="E6:E19">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1535,7 +1541,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1567,7 +1573,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>60.34</v>
+        <v>59.01</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1585,7 +1591,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>60.05</v>
+        <v>58.4</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1603,7 +1609,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>59.45</v>
+        <v>59.7</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1621,7 +1627,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>59.58</v>
+        <v>58.6</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1639,7 +1645,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>56.84</v>
+        <v>57.19</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>39.48</v>
+        <v>39.91</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1670,7 +1676,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>37.04</v>
+        <v>37.6</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1683,7 +1689,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>38.25</v>
+        <v>38.75</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1696,7 +1702,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>58.23</v>
+        <v>58.58</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1709,7 +1715,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>42.55</v>
+        <v>42.88</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1722,7 +1728,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>29.58</v>
+        <v>29.84</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1761,7 +1767,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E19</f>
+        <f>MIBGAS_Spot!E20</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-14
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E20</f>
+        <f>E21</f>
         <v/>
       </c>
     </row>
@@ -1111,10 +1111,10 @@
       <c r="B19" s="12" t="n">
         <v>25.5</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="13" t="n">
         <v>46248</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="12" t="n">
         <v>60.77</v>
       </c>
     </row>
@@ -1125,14 +1125,11 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E20" s="21">
-        <f>AVERAGE(E6:E19)</f>
-        <v/>
+      <c r="D20" s="18" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>60.81</v>
       </c>
     </row>
     <row r="21">
@@ -1142,10 +1139,14 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E21" s="21">
+        <f>AVERAGE(E6:E20)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1155,6 +1156,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1468,12 +1474,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D21:H21"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1483,7 +1489,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E19">
+  <conditionalFormatting sqref="E6:E20">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1541,7 +1547,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1573,7 +1579,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>59.01</v>
+        <v>61.35</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1591,7 +1597,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>58.4</v>
+        <v>60.03</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1609,7 +1615,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>59.7</v>
+        <v>59.95</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1627,7 +1633,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>58.6</v>
+        <v>60.19</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1645,7 +1651,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>57.19</v>
+        <v>56.46</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1663,7 +1669,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>39.91</v>
+        <v>39.93</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1676,7 +1682,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>37.6</v>
+        <v>37.54</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1689,7 +1695,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>38.75</v>
+        <v>38.73</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1702,7 +1708,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>58.58</v>
+        <v>58.7</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1715,7 +1721,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>42.88</v>
+        <v>43.5</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1728,7 +1734,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>29.84</v>
+        <v>29.9</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1767,7 +1773,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E20</f>
+        <f>MIBGAS_Spot!E21</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-15
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E21</f>
+        <f>E22</f>
         <v/>
       </c>
     </row>
@@ -1125,10 +1125,10 @@
       <c r="B20" s="12" t="n">
         <v>26.72</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="13" t="n">
         <v>46249</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="12" t="n">
         <v>60.81</v>
       </c>
     </row>
@@ -1139,14 +1139,11 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E21" s="21">
-        <f>AVERAGE(E6:E20)</f>
-        <v/>
+      <c r="D21" s="18" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>62.41</v>
       </c>
     </row>
     <row r="22">
@@ -1156,10 +1153,14 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E22" s="21">
+        <f>AVERAGE(E6:E21)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1168,6 +1169,11 @@
       </c>
       <c r="B23" s="12" t="n">
         <v>34.55</v>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1478,8 +1484,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D22:H22"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1489,7 +1495,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E20">
+  <conditionalFormatting sqref="E6:E21">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1773,7 +1779,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E21</f>
+        <f>MIBGAS_Spot!E22</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-16
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E22</f>
+        <f>E23</f>
         <v/>
       </c>
     </row>
@@ -1139,10 +1139,10 @@
       <c r="B21" s="12" t="n">
         <v>29.21</v>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="13" t="n">
         <v>46250</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="12" t="n">
         <v>62.41</v>
       </c>
     </row>
@@ -1153,14 +1153,11 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E22" s="21">
-        <f>AVERAGE(E6:E21)</f>
-        <v/>
+      <c r="D22" s="18" t="n">
+        <v>46251</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>63.46</v>
       </c>
     </row>
     <row r="23">
@@ -1170,10 +1167,14 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E23" s="21">
+        <f>AVERAGE(E6:E22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1182,6 +1183,11 @@
       </c>
       <c r="B24" s="12" t="n">
         <v>32.42</v>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1482,9 +1488,9 @@
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
+    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D23:H23"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1495,7 +1501,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E21">
+  <conditionalFormatting sqref="E6:E22">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1779,7 +1785,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E22</f>
+        <f>MIBGAS_Spot!E23</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-17
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E23</f>
+        <f>E24</f>
         <v/>
       </c>
     </row>
@@ -1153,10 +1153,10 @@
       <c r="B22" s="12" t="n">
         <v>31.84</v>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="13" t="n">
         <v>46251</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="12" t="n">
         <v>63.46</v>
       </c>
     </row>
@@ -1167,14 +1167,11 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E23" s="21">
-        <f>AVERAGE(E6:E22)</f>
-        <v/>
+      <c r="D23" s="18" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>61.77</v>
       </c>
     </row>
     <row r="24">
@@ -1184,10 +1181,14 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E24" s="21">
+        <f>AVERAGE(E6:E23)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1197,6 +1198,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1487,8 +1493,8 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
-    <mergeCell ref="D24:H24"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
@@ -1501,7 +1507,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E22">
+  <conditionalFormatting sqref="E6:E23">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1559,7 +1565,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46248</v>
+        <v>46251</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1591,7 +1597,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>61.35</v>
+        <v>62.03</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1609,7 +1615,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>60.03</v>
+        <v>60.7</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1627,7 +1633,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>59.95</v>
+        <v>60.53</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1645,7 +1651,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>60.19</v>
+        <v>60.5</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1663,7 +1669,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>56.46</v>
+        <v>57.63</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1681,7 +1687,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>39.93</v>
+        <v>40.19</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1694,7 +1700,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>37.54</v>
+        <v>37.83</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1707,7 +1713,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>38.73</v>
+        <v>39</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1720,7 +1726,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>58.7</v>
+        <v>59.08</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1733,7 +1739,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>43.5</v>
+        <v>43.23</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1746,7 +1752,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>29.9</v>
+        <v>30.08</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1785,7 +1791,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E23</f>
+        <f>MIBGAS_Spot!E24</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-18
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E24</f>
+        <f>E25</f>
         <v/>
       </c>
     </row>
@@ -1167,10 +1167,10 @@
       <c r="B23" s="12" t="n">
         <v>34.55</v>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="13" t="n">
         <v>46252</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="12" t="n">
         <v>61.77</v>
       </c>
     </row>
@@ -1181,14 +1181,11 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E24" s="21">
-        <f>AVERAGE(E6:E23)</f>
-        <v/>
+      <c r="D24" s="18" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>63.61</v>
       </c>
     </row>
     <row r="25">
@@ -1198,10 +1195,14 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E25" s="21">
+        <f>AVERAGE(E6:E24)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -1211,6 +1212,11 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1493,11 +1499,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D25:H25"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1507,7 +1513,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E23">
+  <conditionalFormatting sqref="E6:E24">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1565,7 +1571,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1597,7 +1603,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>62.03</v>
+        <v>62.34</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1615,7 +1621,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>60.7</v>
+        <v>62.65</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1633,7 +1639,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>60.53</v>
+        <v>62.73</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>60.5</v>
+        <v>61.65</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1669,7 +1675,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>57.63</v>
+        <v>59.87</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>40.19</v>
+        <v>41.34</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1700,7 +1706,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>37.83</v>
+        <v>38.94</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1713,7 +1719,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>39</v>
+        <v>40.13</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1726,7 +1732,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>59.08</v>
+        <v>61.31</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1739,7 +1745,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>43.23</v>
+        <v>44.63</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1752,7 +1758,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>30.08</v>
+        <v>30.68</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1791,7 +1797,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E24</f>
+        <f>MIBGAS_Spot!E25</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-19
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E25</f>
+        <f>E26</f>
         <v/>
       </c>
     </row>
@@ -1181,10 +1181,10 @@
       <c r="B24" s="12" t="n">
         <v>32.42</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="13" t="n">
         <v>46253</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="12" t="n">
         <v>63.61</v>
       </c>
     </row>
@@ -1195,14 +1195,11 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E25" s="21">
-        <f>AVERAGE(E6:E24)</f>
-        <v/>
+      <c r="D25" s="18" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>63.47</v>
       </c>
     </row>
     <row r="26">
@@ -1212,10 +1209,14 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E26" s="21">
+        <f>AVERAGE(E6:E25)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1224,6 +1225,11 @@
       </c>
       <c r="B27" s="12" t="n">
         <v>40.41</v>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1502,8 +1508,8 @@
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D27:H27"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D26:H26"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1513,7 +1519,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E24">
+  <conditionalFormatting sqref="E6:E25">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1571,7 +1577,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1603,7 +1609,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>62.34</v>
+        <v>62.97</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1621,7 +1627,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>62.65</v>
+        <v>62.2</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1639,7 +1645,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>62.73</v>
+        <v>62.25</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1657,7 +1663,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>61.65</v>
+        <v>62.35</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1675,7 +1681,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>59.87</v>
+        <v>59.84</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1693,7 +1699,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>41.34</v>
+        <v>41.74</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1706,7 +1712,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>38.94</v>
+        <v>39.26</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1719,7 +1725,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>40.13</v>
+        <v>40.49</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1732,7 +1738,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>61.31</v>
+        <v>61.1</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1745,7 +1751,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>44.63</v>
+        <v>44.88</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1758,7 +1764,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>30.68</v>
+        <v>30.78</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1797,7 +1803,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E25</f>
+        <f>MIBGAS_Spot!E26</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-20
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -154,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -203,12 +203,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1195,10 +1189,10 @@
       <c r="B25" s="12" t="n">
         <v>38.45</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="13" t="n">
         <v>46254</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="12" t="n">
         <v>63.47</v>
       </c>
     </row>
@@ -1209,12 +1203,12 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>MEDIA MES</t>
         </is>
       </c>
-      <c r="E26" s="21">
+      <c r="E26" s="19">
         <f>AVERAGE(E6:E25)</f>
         <v/>
       </c>
@@ -1226,7 +1220,7 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
         </is>
@@ -1404,103 +1398,103 @@
       <c r="A49" s="11" t="n">
         <v>46235</v>
       </c>
-      <c r="B49" s="23" t="n"/>
+      <c r="B49" s="21" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
         <v>46266</v>
       </c>
-      <c r="B50" s="23" t="n"/>
+      <c r="B50" s="21" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
         <v>46296</v>
       </c>
-      <c r="B51" s="23" t="n"/>
+      <c r="B51" s="21" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
         <v>46327</v>
       </c>
-      <c r="B52" s="23" t="n"/>
+      <c r="B52" s="21" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
         <v>46357</v>
       </c>
-      <c r="B53" s="23" t="n"/>
+      <c r="B53" s="21" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
         <v>46388</v>
       </c>
-      <c r="B54" s="23" t="n"/>
+      <c r="B54" s="21" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
         <v>46419</v>
       </c>
-      <c r="B55" s="23" t="n"/>
+      <c r="B55" s="21" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
         <v>46447</v>
       </c>
-      <c r="B56" s="23" t="n"/>
+      <c r="B56" s="21" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
         <v>46478</v>
       </c>
-      <c r="B57" s="23" t="n"/>
+      <c r="B57" s="21" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
         <v>46508</v>
       </c>
-      <c r="B58" s="23" t="n"/>
+      <c r="B58" s="21" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
         <v>46539</v>
       </c>
-      <c r="B59" s="23" t="n"/>
+      <c r="B59" s="21" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
         <v>46569</v>
       </c>
-      <c r="B60" s="23" t="n"/>
+      <c r="B60" s="21" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
         <v>46600</v>
       </c>
-      <c r="B61" s="23" t="n"/>
+      <c r="B61" s="21" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
         <v>46631</v>
       </c>
-      <c r="B62" s="23" t="n"/>
+      <c r="B62" s="21" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
         <v>46661</v>
       </c>
-      <c r="B63" s="23" t="n"/>
+      <c r="B63" s="21" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
         <v>46692</v>
       </c>
-      <c r="B64" s="23" t="n"/>
+      <c r="B64" s="21" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
         <v>46722</v>
       </c>
-      <c r="B65" s="23" t="n"/>
+      <c r="B65" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1571,12 +1565,12 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Fecha de la curva:</t>
         </is>
       </c>
-      <c r="B4" s="25" t="n">
+      <c r="B4" s="23" t="n">
         <v>46253</v>
       </c>
     </row>
@@ -1603,217 +1597,217 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Mes M+1 (Sep26-Sep26)</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="25" t="n">
         <v>62.97</v>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>· Forward &gt; spot (contango): el mercado espera gas más caro — renovar pronto y revisar fijaciones.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Mes M+2 (Oct26-Oct26)</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="25" t="n">
         <v>62.2</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>· Forward &lt; spot (backwardation): el mercado espera relajación — favorece indexado y esperar.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Mes M+3 (Nov26-Nov26)</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="25" t="n">
         <v>62.25</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>· Estacionalidad estructural: el invierno (GSES_W) cotiza por encima del verano (GSES_S). Un fijo anual promedia las dos.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+1 (Oct26-Dec26)</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="25" t="n">
         <v>62.35</v>
       </c>
-      <c r="C9" s="28" t="n">
+      <c r="C9" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>· Control de plausibilidad de ofertas (ficha de gas): energía sin peajes esperada ≈ forward + 15-25 €/MWh de margen.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+2 (Jan27-Mar27)</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="25" t="n">
         <v>59.84</v>
       </c>
-      <c r="C10" s="28" t="n">
+      <c r="C10" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>· El precio TUR de materia prima se referencia a MIBGAS: esta curva ANTICIPA los reprecios trimestrales de la TUR (ene/abr/jul/oct).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+3 (Apr27-Jun27)</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="25" t="n">
         <v>41.74</v>
       </c>
-      <c r="C11" s="28" t="n">
+      <c r="C11" s="26" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Trimestre Q+4 (Jul27-Sep27)</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="25" t="n">
         <v>39.26</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="26" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Verano (abr-sep) (Apr27-Sep27)</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="25" t="n">
         <v>40.49</v>
       </c>
-      <c r="C13" s="28" t="n">
+      <c r="C13" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Invierno (oct-mar) (Oct26-Mar27)</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n">
+      <c r="B14" s="25" t="n">
         <v>61.1</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Año Y+1 (Jan27-Dec27)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n">
+      <c r="B15" s="25" t="n">
         <v>44.88</v>
       </c>
-      <c r="C15" s="28" t="n">
+      <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Año Y+2 (Jan28-Dec28)</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="25" t="n">
         <v>30.78</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suma de pesos (debe ser 12)</t>
         </is>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <f>SUM(C6:C16)</f>
         <v/>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="22">
         <f>IF(B18=12,"OK","⚠")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="34" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>FORWARD PRÓXIMOS 12 MESES (€/MWh)</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="33">
         <f>SUMPRODUCT(B6:B16,C6:C16)/SUM(C6:C16)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Spot del mes en curso (€/MWh)</t>
         </is>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="31">
         <f>MIBGAS_Spot!E26</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Contango/backwardation (forward − spot)</t>
         </is>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="31">
         <f>B19-B20</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-21
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E27</f>
+        <f>E28</f>
         <v/>
       </c>
     </row>
@@ -1209,10 +1209,10 @@
       <c r="B26" s="12" t="n">
         <v>36.68</v>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="13" t="n">
         <v>46255</v>
       </c>
-      <c r="E26" s="19" t="n">
+      <c r="E26" s="12" t="n">
         <v>65.61</v>
       </c>
     </row>
@@ -1223,14 +1223,11 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E27" s="21">
-        <f>AVERAGE(E6:E26)</f>
-        <v/>
+      <c r="D27" s="18" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>66.31</v>
       </c>
     </row>
     <row r="28">
@@ -1240,10 +1237,14 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E28" s="21">
+        <f>AVERAGE(E6:E27)</f>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1252,6 +1253,11 @@
       </c>
       <c r="B29" s="12" t="n">
         <v>46.23</v>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1513,8 +1519,8 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="D28:H28"/>
     <mergeCell ref="A2:H3"/>
+    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1525,7 +1531,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E26">
+  <conditionalFormatting sqref="E6:E27">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1583,7 +1589,7 @@
         </is>
       </c>
       <c r="B4" s="25" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
@@ -1615,7 +1621,7 @@
         </is>
       </c>
       <c r="B6" s="27" t="n">
-        <v>64.48999999999999</v>
+        <v>66.04000000000001</v>
       </c>
       <c r="C6" s="28" t="n">
         <v>1</v>
@@ -1633,7 +1639,7 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>62.96</v>
+        <v>65.25</v>
       </c>
       <c r="C7" s="28" t="n">
         <v>0</v>
@@ -1651,7 +1657,7 @@
         </is>
       </c>
       <c r="B8" s="27" t="n">
-        <v>64.2</v>
+        <v>66.25</v>
       </c>
       <c r="C8" s="28" t="n">
         <v>0</v>
@@ -1669,7 +1675,7 @@
         </is>
       </c>
       <c r="B9" s="27" t="n">
-        <v>64.25</v>
+        <v>65.87</v>
       </c>
       <c r="C9" s="28" t="n">
         <v>3</v>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>61.66</v>
+        <v>63.75</v>
       </c>
       <c r="C10" s="28" t="n">
         <v>3</v>
@@ -1705,7 +1711,7 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>43.34</v>
+        <v>44.88</v>
       </c>
       <c r="C11" s="28" t="n">
         <v>3</v>
@@ -1718,7 +1724,7 @@
         </is>
       </c>
       <c r="B12" s="27" t="n">
-        <v>40.69</v>
+        <v>42.01</v>
       </c>
       <c r="C12" s="28" t="n">
         <v>2</v>
@@ -1731,7 +1737,7 @@
         </is>
       </c>
       <c r="B13" s="27" t="n">
-        <v>42.01</v>
+        <v>43.44</v>
       </c>
       <c r="C13" s="28" t="n">
         <v>0</v>
@@ -1744,7 +1750,7 @@
         </is>
       </c>
       <c r="B14" s="27" t="n">
-        <v>62.96</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="C14" s="28" t="n">
         <v>0</v>
@@ -1757,7 +1763,7 @@
         </is>
       </c>
       <c r="B15" s="27" t="n">
-        <v>46.15</v>
+        <v>47.95</v>
       </c>
       <c r="C15" s="28" t="n">
         <v>0</v>
@@ -1770,7 +1776,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>31.48</v>
+        <v>32.4</v>
       </c>
       <c r="C16" s="28" t="n">
         <v>0</v>
@@ -1809,7 +1815,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E27</f>
+        <f>MIBGAS_Spot!E28</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Radar: datos de 2026-08-22
</commit_message>
<xml_diff>
--- a/excel/ACZO_Radar_Gas.xlsx
+++ b/excel/ACZO_Radar_Gas.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="K18" s="17">
-        <f>E28</f>
+        <f>E29</f>
         <v/>
       </c>
     </row>
@@ -1223,10 +1223,10 @@
       <c r="B27" s="12" t="n">
         <v>40.41</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="13" t="n">
         <v>46256</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E27" s="12" t="n">
         <v>66.31</v>
       </c>
     </row>
@@ -1237,14 +1237,11 @@
       <c r="B28" s="12" t="n">
         <v>44.16</v>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>MEDIA MES</t>
-        </is>
-      </c>
-      <c r="E28" s="21">
-        <f>AVERAGE(E6:E27)</f>
-        <v/>
+      <c r="D28" s="18" t="n">
+        <v>46257</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>66.68000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1254,10 +1251,14 @@
       <c r="B29" s="12" t="n">
         <v>46.23</v>
       </c>
-      <c r="D29" s="22" t="inlineStr">
-        <is>
-          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
-        </is>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>MEDIA MES</t>
+        </is>
+      </c>
+      <c r="E29" s="21">
+        <f>AVERAGE(E6:E28)</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1267,6 +1268,11 @@
       <c r="B30" s="12" t="n">
         <v>48.47</v>
       </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Filas naranjas = entregas futuras ya cotizadas (mañana, pasado).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -1516,11 +1522,11 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="D30:H30"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="A4"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:H3"/>
-    <mergeCell ref="D29:H29"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:B65">
@@ -1531,7 +1537,7 @@
       <formula>AND(ISNUMBER($B6),$B6&gt;=$B$4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E27">
+  <conditionalFormatting sqref="E6:E28">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>AND(ISNUMBER(E6),E6&lt;$B$4)</formula>
     </cfRule>
@@ -1815,7 +1821,7 @@
         </is>
       </c>
       <c r="B20" s="33">
-        <f>MIBGAS_Spot!E28</f>
+        <f>MIBGAS_Spot!E29</f>
         <v/>
       </c>
     </row>

</xml_diff>